<commit_message>
feat(siakred): pilih RPS MK penciri dari RPS SI-OBE (tanpa unggah ulang)
- Panel "Pilih Mata Kuliah Penciri" di Detail Butir ber-kode bersama
  PRODI-RPS-MK-PENCIRI (LAMSPAK Unggul: U2.02 & U5.10) untuk akun prodi/superadmin
- Tiap MK terpilih jadi dokumen cermin yang memakai file RPS yang sama
  (tanpa salinan), verifikasi APPROVED; batal pilih -> diarsipkan
- Sinkron malam memperbarui cermin saat RPS sumber direvisi / dicabut
- Data LAMSPAK Unggul: kode bersama U2.02/U5.10 + panduan butir RPS

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/master_akreditasi/data/LAMSPAK-UNGGUL_import.xlsx
+++ b/master_akreditasi/data/LAMSPAK-UNGGUL_import.xlsx
@@ -2066,7 +2066,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Dokumen bersama dengan butir U5.09 (Standar 5): cukup diunggah sekali di salah satu butir, otomatis terhitung di keduanya.</t>
+          <t>Tidak perlu unggah: RPS yang disahkan di SI-OBE masuk otomatis (1 dokumen per MK). Berlaku juga untuk butir U5.09.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2119,8 +2119,16 @@
           <t>Bukti kedalaman dan keluasan pembelajaran bidang keilmuan program studi</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Tidak perlu unggah: pilih MK penciri dari RPS yang sudah disahkan di SI-OBE pada halaman butir ini. Berlaku juga untuk butir U5.10.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>PRODI-RPS-MK-PENCIRI</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4970,7 +4978,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Dokumen bersama dengan butir U2.01 (Standar 2): cukup diunggah sekali di salah satu butir, otomatis terhitung di keduanya.</t>
+          <t>Tidak perlu unggah: RPS yang disahkan di SI-OBE masuk otomatis (1 dokumen per MK). Berlaku juga untuk butir U2.01.</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -5023,8 +5031,16 @@
           <t>Bukti kekhasan keilmuan program studi</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Tidak perlu unggah: pilih MK penciri dari RPS yang sudah disahkan di SI-OBE pada halaman butir ini. Berlaku juga untuk butir U2.02.</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>PRODI-RPS-MK-PENCIRI</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">

</xml_diff>

<commit_message>
feat(siakred): tautan SIAMI (U11.22) & SIAKUN input nilai (U3.14)
- isi_tautan_aplikasi: + SIAMI (siami.unisan-g.id) & SIAKUN untuk input nilai
- U3.14 diberi kode bersama PRODI-SCREENSHOT-INPUT-NILAI-SIAKAD
- Dokumen Saya: dokumen umum (scope kosong) ikut terhitung di butir PRODI/FAKULTAS,
  sama dengan aturan halaman Sesi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/master_akreditasi/data/LAMSPAK-UNGGUL_import.xlsx
+++ b/master_akreditasi/data/LAMSPAK-UNGGUL_import.xlsx
@@ -3554,7 +3554,11 @@
         </is>
       </c>
       <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>PRODI-SCREENSHOT-INPUT-NILAI-SIAKAD</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">

</xml_diff>